<commit_message>
fix: Add processing pattern assignments for libraries and development-tools
Investigated ALL 105 files (49 libraries + 56 development-tools) and added
Processing Pattern (PP) assignments to 17 pattern-specific files:

Libraries (1 file):
- jaxrs_access_log.rst → PP=restful-web-service

Development-tools Testing Framework (16 files):
- batch.rst (2 files) → PP=nablarch-batch
- rest.rst (2 files) → PP=restful-web-service
- MOM messaging tests (8 files) → PP=mom-messaging
- HTTP messaging tests (4 files) → PP=http-messaging

Updated classification rules in both classification.md and generate-mapping.py
to enable category-based filtering for knowledge file generation.

This addresses reviewer feedback: "全ての中身を見て処理パターンを判断する必要があります"

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.claude/skills/nabledge-creator/output/mapping-v6.xlsx
+++ b/.claude/skills/nabledge-creator/output/mapping-v6.xlsx
@@ -6638,7 +6638,11 @@
           <t>libraries</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>restful-web-service</t>
+        </is>
+      </c>
       <c r="H156" t="inlineStr">
         <is>
           <t>component/libraries/log/jaxrs-access-log.json</t>
@@ -10308,7 +10312,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>nablarch-batch</t>
+        </is>
+      </c>
       <c r="H247" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/batch.json</t>
@@ -10346,7 +10354,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr"/>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H248" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/delayed-receive.json</t>
@@ -10384,7 +10396,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H249" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/delayed-send.json</t>
@@ -10494,7 +10510,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr"/>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>http-messaging</t>
+        </is>
+      </c>
       <c r="H252" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/http-real.json</t>
@@ -10532,7 +10552,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>http-messaging</t>
+        </is>
+      </c>
       <c r="H253" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/http-send-sync.json</t>
@@ -10646,7 +10670,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr"/>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H256" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/real.json</t>
@@ -10684,7 +10712,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr"/>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>restful-web-service</t>
+        </is>
+      </c>
       <c r="H257" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/rest.json</t>
@@ -10722,7 +10754,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G258" t="inlineStr"/>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H258" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/02_RequestUnitTest/send-sync.json</t>
@@ -10760,7 +10796,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G259" t="inlineStr"/>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>nablarch-batch</t>
+        </is>
+      </c>
       <c r="H259" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/batch.json</t>
@@ -10798,7 +10838,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H260" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/delayed-receive.json</t>
@@ -10836,7 +10880,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr"/>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H261" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/delayed-send.json</t>
@@ -10874,7 +10922,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr"/>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>http-messaging</t>
+        </is>
+      </c>
       <c r="H262" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/http-send-sync.json</t>
@@ -10950,7 +11002,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr"/>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H264" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/real.json</t>
@@ -10988,7 +11044,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>restful-web-service</t>
+        </is>
+      </c>
       <c r="H265" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/rest.json</t>
@@ -11026,7 +11086,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr"/>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H266" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/05_UnitTestGuide/03_DealUnitTest/send-sync.json</t>
@@ -11368,7 +11432,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G275" t="inlineStr"/>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>http-messaging</t>
+        </is>
+      </c>
       <c r="H275" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/06_TestFWGuide/RequestUnitTest-http-send-sync.json</t>
@@ -11406,7 +11474,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr"/>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H276" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/06_TestFWGuide/RequestUnitTest-real.json</t>
@@ -11482,7 +11554,11 @@
           <t>testing-framework</t>
         </is>
       </c>
-      <c r="G278" t="inlineStr"/>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>mom-messaging</t>
+        </is>
+      </c>
       <c r="H278" t="inlineStr">
         <is>
           <t>development-tools/testing-framework/06_TestFWGuide/RequestUnitTest-send-sync.json</t>

</xml_diff>